<commit_message>
Final version of ILOptim.xlsx
</commit_message>
<xml_diff>
--- a/WebPWrapperLib/ILOptim.xlsx
+++ b/WebPWrapperLib/ILOptim.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\Administrator\source\repos\repzilon\WebP-wrapper-animatedWebP\WebPWrapperLib\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BE641F5-78C9-454E-928B-415704C319DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E422F6-A68A-4C3C-9A8E-6AE60F7E1979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10170" yWindow="3945" windowWidth="17235" windowHeight="12735" xr2:uid="{799CC530-1EA5-40BE-81F2-E7ECAB72BC1F}"/>
   </bookViews>
@@ -1012,6 +1012,24 @@
       <c r="E18">
         <v>1</v>
       </c>
+      <c r="F18">
+        <v>104</v>
+      </c>
+      <c r="G18">
+        <v>2</v>
+      </c>
+      <c r="H18">
+        <v>2</v>
+      </c>
+      <c r="I18">
+        <v>104</v>
+      </c>
+      <c r="J18">
+        <v>2</v>
+      </c>
+      <c r="K18">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>